<commit_message>
Lead ILLUCO mirror listings with the first-look clarity message
Sales team feedback: people are wowed the moment they look into the
mirror. Titles now say UHD (ILLUCO's own term on illuco.com), bullet 1
and the description open with "see the difference at first look"
(99% vs 60-70% reflectance, over 40% brighter), and backend keywords
add "hd high definition". Notes workbook regenerated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JtZ82rKJM1p58HzVJpKZqv
</commit_message>
<xml_diff>
--- a/CRL DOC/ILLUCO/ILLUCO_Upload_Notes.xlsx
+++ b/CRL DOC/ILLUCO/ILLUCO_Upload_Notes.xlsx
@@ -1244,22 +1244,22 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>ILLUCO Dental Mirrors with Handles, Grand Size 10 (34mm) and Double-Sided Size 4 (22mm), Front Surface Dielectric Mouth Mirror, 99% Reflectance, Fog-Resistant, Autoclavable 100X</t>
+          <t>ILLUCO UHD Dental Mirrors with Handles, Grand Size 10 (34mm) and Double-Sided Size 4 (22mm), Front Surface Dielectric Mouth Mirror, 99% Reflectance, Fog-Resistant, Autoclavable 100X</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
+          <t>SEE THE DIFFERENCE AT FIRST LOOK: Most dental mirrors reflect only 60-70% of light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, for an image over 40% brighter, crisp, true to color and free of ghosting. Look into it once and you will notice it.</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
           <t>TWO NEW ILLUCO MIRRORS: Grand Size 10 (34mm) in 1X or 2X for a 2.4x wider field of view, and Double-Sided Size 4 (22mm) with 99% reflectance on both faces.</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>99% REFLECTANCE, ZERO GHOST IMAGES: Front surface dielectric coating on German optical glass for a bright, sharp, distortion-free image.</t>
-        </is>
-      </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>FOG-RESISTANT: Water-repellent coating sheds saliva and spray mid-procedure.</t>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>ILLUCO front surface dielectric dental mirrors deliver 99% reflectance, no ghost images and a fog-resistant, water-repellent surface that withstands 100 autoclave cycles. Choose the Grand Size 10 (34mm) mirror in 1X or 2X for a 2.4x wider field of view, or the Double-Sided Size 4 (22mm) mirror with 99% reflectance on both faces. Each kit includes ergonomic anti-rotation handles in Light Blue or Dark Blue. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C).</t>
+          <t>The first thing dental professionals notice about an ILLUCO mirror is the view. Most dental mirrors reflect only 60-70% of available light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, so the image is over 40% brighter, sharp, true to color and free of the ghost images that cause visual fatigue. You see the difference the moment you look into it. The fog-resistant, water-repellent surface withstands 100 autoclave cycles. Choose the Grand Size 10 (34mm) mirror in 1X or 2X for a 2.4x wider field of view, or the Double-Sided Size 4 (22mm) mirror with 99% reflectance on both faces. Each kit includes ergonomic anti-rotation handles in Light Blue or Dark Blue. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C).</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
@@ -1297,22 +1297,22 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>ILLUCO Grand Dental Mirror Size 10 (34mm) with Handles, 2 Pack, Large Front Surface Mouth Mirror, 99% Reflectance, Fog-Resistant, Autoclavable 100X, No Ghost Image (1X, Light Blue)</t>
+          <t>ILLUCO Grand UHD Dental Mirror Size 10 (34mm) with Handles, 2 Pack, Large Front Surface Mouth Mirror, 99% Reflectance, Fog-Resistant, Autoclavable 100X, No Ghost Image (1X, Light Blue)</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
+          <t>SEE THE DIFFERENCE AT FIRST LOOK: Most dental mirrors reflect only 60-70% of light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, for an image over 40% brighter, crisp, true to color and free of ghosting. Look into it once and you will notice it.</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
           <t>2.4X WIDER FIELD OF VIEW: The Size 10 (34mm) head covers 2.4 times the viewing area of a standard Size 4 (22mm) mirror. See a full quadrant, multi-unit restorations or the whole arch in one view, with far less mirror repositioning.</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>99% REFLECTANCE, ZERO GHOST IMAGES: Front surface dielectric coating on German optical glass reflects 99% of light vs 60-70% for standard mirrors, for a bright, sharp, distortion-free image with no secondary reflection.</t>
-        </is>
-      </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
           <t>ATRAUMATIC RETRACTION, MORE LIGHT: The broad 34mm head spreads pressure for comfortable cheek and tongue retraction in oral surgery, periodontics and orthodontic checks, and bounces more operatory light into dark posterior regions.</t>
@@ -1330,16 +1330,16 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The ILLUCO Grand Dental Mirror scales the standard mouth mirror up to a Size 10 (34mm) head, giving a 2.4x wider field of view than a standard Size 4 (22mm) mirror. View an entire quadrant, multi-unit restorations or full-arch alignment in a single glance and spend less time repositioning. The wide 34mm surface also distributes pressure evenly for comfortable cheek and tongue retraction, and works as a reflector that bounces more overhead light into deep posterior regions. ILLUCO's front surface dielectric coating on German optical glass reflects 99% of available light, compared with 60-70% for standard mirrors, and eliminates the ghost images that cause visual fatigue. The surface is large and distortion-free enough for clean quadrant photos. A water-repellent coating keeps the view clear mid-procedure, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each kit includes 2 Grand Size 10 mirror heads, 2 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in 1X and 2X magnification, Light Blue and Dark Blue.</t>
+          <t>The first thing dental professionals notice about an ILLUCO mirror is the view. Most dental mirrors reflect only 60-70% of available light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, so the image is over 40% brighter, sharp, true to color and free of the ghost images that cause visual fatigue. You see the difference the moment you look into it. The ILLUCO Grand Dental Mirror puts that clarity on a Size 10 (34mm) head, giving a 2.4x wider field of view than a standard Size 4 (22mm) mirror. View an entire quadrant, multi-unit restorations or full-arch alignment in a single glance and spend less time repositioning. The wide 34mm surface also distributes pressure evenly for comfortable cheek and tongue retraction, and works as a reflector that bounces more overhead light into deep posterior regions. The surface is large and distortion-free enough for clean quadrant photos. A water-repellent coating keeps the view clear mid-procedure, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each kit includes 2 Grand Size 10 mirror heads, 2 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in 1X and 2X magnification, Light Blue and Dark Blue.</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>large mouth mirror oversize jumbo wide view dentist orthodontist oral surgery retractor intraoral photography quadrant dental tools dentist instruments tooth teeth oral exam anti fog hygienist magnifying 2x</t>
+          <t>large mouth mirror oversize jumbo wide view dentist orthodontist oral surgery retractor intraoral photography quadrant dental tools dentist instruments tooth teeth oral exam anti fog hygienist magnifying 2x hd high definition</t>
         </is>
       </c>
       <c r="K3" s="3" t="n">
-        <v>206</v>
+        <v>225</v>
       </c>
     </row>
     <row r="4">
@@ -1350,22 +1350,22 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>ILLUCO Grand Dental Mirror Size 10 (34mm) with Handles, 2 Pack, Large Front Surface Mouth Mirror, 99% Reflectance, Fog-Resistant, Autoclavable 100X, No Ghost Image (1X, Dark Blue)</t>
+          <t>ILLUCO Grand UHD Dental Mirror Size 10 (34mm) with Handles, 2 Pack, Large Front Surface Mouth Mirror, 99% Reflectance, Fog-Resistant, Autoclavable 100X, No Ghost Image (1X, Dark Blue)</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
+          <t>SEE THE DIFFERENCE AT FIRST LOOK: Most dental mirrors reflect only 60-70% of light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, for an image over 40% brighter, crisp, true to color and free of ghosting. Look into it once and you will notice it.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
           <t>2.4X WIDER FIELD OF VIEW: The Size 10 (34mm) head covers 2.4 times the viewing area of a standard Size 4 (22mm) mirror. See a full quadrant, multi-unit restorations or the whole arch in one view, with far less mirror repositioning.</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>99% REFLECTANCE, ZERO GHOST IMAGES: Front surface dielectric coating on German optical glass reflects 99% of light vs 60-70% for standard mirrors, for a bright, sharp, distortion-free image with no secondary reflection.</t>
-        </is>
-      </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
           <t>ATRAUMATIC RETRACTION, MORE LIGHT: The broad 34mm head spreads pressure for comfortable cheek and tongue retraction in oral surgery, periodontics and orthodontic checks, and bounces more operatory light into dark posterior regions.</t>
@@ -1383,16 +1383,16 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The ILLUCO Grand Dental Mirror scales the standard mouth mirror up to a Size 10 (34mm) head, giving a 2.4x wider field of view than a standard Size 4 (22mm) mirror. View an entire quadrant, multi-unit restorations or full-arch alignment in a single glance and spend less time repositioning. The wide 34mm surface also distributes pressure evenly for comfortable cheek and tongue retraction, and works as a reflector that bounces more overhead light into deep posterior regions. ILLUCO's front surface dielectric coating on German optical glass reflects 99% of available light, compared with 60-70% for standard mirrors, and eliminates the ghost images that cause visual fatigue. The surface is large and distortion-free enough for clean quadrant photos. A water-repellent coating keeps the view clear mid-procedure, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each kit includes 2 Grand Size 10 mirror heads, 2 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in 1X and 2X magnification, Light Blue and Dark Blue.</t>
+          <t>The first thing dental professionals notice about an ILLUCO mirror is the view. Most dental mirrors reflect only 60-70% of available light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, so the image is over 40% brighter, sharp, true to color and free of the ghost images that cause visual fatigue. You see the difference the moment you look into it. The ILLUCO Grand Dental Mirror puts that clarity on a Size 10 (34mm) head, giving a 2.4x wider field of view than a standard Size 4 (22mm) mirror. View an entire quadrant, multi-unit restorations or full-arch alignment in a single glance and spend less time repositioning. The wide 34mm surface also distributes pressure evenly for comfortable cheek and tongue retraction, and works as a reflector that bounces more overhead light into deep posterior regions. The surface is large and distortion-free enough for clean quadrant photos. A water-repellent coating keeps the view clear mid-procedure, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each kit includes 2 Grand Size 10 mirror heads, 2 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in 1X and 2X magnification, Light Blue and Dark Blue.</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>large mouth mirror oversize jumbo wide view dentist orthodontist oral surgery retractor intraoral photography quadrant dental tools dentist instruments tooth teeth oral exam anti fog hygienist magnifying 2x</t>
+          <t>large mouth mirror oversize jumbo wide view dentist orthodontist oral surgery retractor intraoral photography quadrant dental tools dentist instruments tooth teeth oral exam anti fog hygienist magnifying 2x hd high definition</t>
         </is>
       </c>
       <c r="K4" s="3" t="n">
-        <v>206</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5">
@@ -1403,22 +1403,22 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>ILLUCO Grand Dental Mirror Size 10 (34mm) with Handles, 2 Pack, Large Front Surface Mouth Mirror, 99% Reflectance, Fog-Resistant, Autoclavable 100X, No Ghost Image (2X, Light Blue)</t>
+          <t>ILLUCO Grand UHD Dental Mirror Size 10 (34mm) with Handles, 2 Pack, Large Front Surface Mouth Mirror, 99% Reflectance, Fog-Resistant, Autoclavable 100X, No Ghost Image (2X, Light Blue)</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
+          <t>SEE THE DIFFERENCE AT FIRST LOOK: Most dental mirrors reflect only 60-70% of light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, for an image over 40% brighter, crisp, true to color and free of ghosting. Look into it once and you will notice it.</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
           <t>2.4X WIDER FIELD OF VIEW: The Size 10 (34mm) head covers 2.4 times the viewing area of a standard Size 4 (22mm) mirror. See a full quadrant, multi-unit restorations or the whole arch in one view, with far less mirror repositioning.</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>99% REFLECTANCE, ZERO GHOST IMAGES: Front surface dielectric coating on German optical glass reflects 99% of light vs 60-70% for standard mirrors, for a bright, sharp, distortion-free image with no secondary reflection.</t>
-        </is>
-      </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
           <t>ATRAUMATIC RETRACTION, MORE LIGHT: The broad 34mm head spreads pressure for comfortable cheek and tongue retraction in oral surgery, periodontics and orthodontic checks, and bounces more operatory light into dark posterior regions.</t>
@@ -1436,16 +1436,16 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The ILLUCO Grand Dental Mirror scales the standard mouth mirror up to a Size 10 (34mm) head, giving a 2.4x wider field of view than a standard Size 4 (22mm) mirror. View an entire quadrant, multi-unit restorations or full-arch alignment in a single glance and spend less time repositioning. The wide 34mm surface also distributes pressure evenly for comfortable cheek and tongue retraction, and works as a reflector that bounces more overhead light into deep posterior regions. ILLUCO's front surface dielectric coating on German optical glass reflects 99% of available light, compared with 60-70% for standard mirrors, and eliminates the ghost images that cause visual fatigue. The surface is large and distortion-free enough for clean quadrant photos. A water-repellent coating keeps the view clear mid-procedure, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each kit includes 2 Grand Size 10 mirror heads, 2 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in 1X and 2X magnification, Light Blue and Dark Blue.</t>
+          <t>The first thing dental professionals notice about an ILLUCO mirror is the view. Most dental mirrors reflect only 60-70% of available light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, so the image is over 40% brighter, sharp, true to color and free of the ghost images that cause visual fatigue. You see the difference the moment you look into it. The ILLUCO Grand Dental Mirror puts that clarity on a Size 10 (34mm) head, giving a 2.4x wider field of view than a standard Size 4 (22mm) mirror. View an entire quadrant, multi-unit restorations or full-arch alignment in a single glance and spend less time repositioning. The wide 34mm surface also distributes pressure evenly for comfortable cheek and tongue retraction, and works as a reflector that bounces more overhead light into deep posterior regions. The surface is large and distortion-free enough for clean quadrant photos. A water-repellent coating keeps the view clear mid-procedure, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each kit includes 2 Grand Size 10 mirror heads, 2 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in 1X and 2X magnification, Light Blue and Dark Blue.</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>large mouth mirror oversize jumbo wide view dentist orthodontist oral surgery retractor intraoral photography quadrant dental tools dentist instruments tooth teeth oral exam anti fog hygienist magnifying 2x</t>
+          <t>large mouth mirror oversize jumbo wide view dentist orthodontist oral surgery retractor intraoral photography quadrant dental tools dentist instruments tooth teeth oral exam anti fog hygienist magnifying 2x hd high definition</t>
         </is>
       </c>
       <c r="K5" s="3" t="n">
-        <v>206</v>
+        <v>225</v>
       </c>
     </row>
     <row r="6">
@@ -1456,22 +1456,22 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>ILLUCO Grand Dental Mirror Size 10 (34mm) with Handles, 2 Pack, Large Front Surface Mouth Mirror, 99% Reflectance, Fog-Resistant, Autoclavable 100X, No Ghost Image (2X, Dark Blue)</t>
+          <t>ILLUCO Grand UHD Dental Mirror Size 10 (34mm) with Handles, 2 Pack, Large Front Surface Mouth Mirror, 99% Reflectance, Fog-Resistant, Autoclavable 100X, No Ghost Image (2X, Dark Blue)</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
+          <t>SEE THE DIFFERENCE AT FIRST LOOK: Most dental mirrors reflect only 60-70% of light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, for an image over 40% brighter, crisp, true to color and free of ghosting. Look into it once and you will notice it.</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
           <t>2.4X WIDER FIELD OF VIEW: The Size 10 (34mm) head covers 2.4 times the viewing area of a standard Size 4 (22mm) mirror. See a full quadrant, multi-unit restorations or the whole arch in one view, with far less mirror repositioning.</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>99% REFLECTANCE, ZERO GHOST IMAGES: Front surface dielectric coating on German optical glass reflects 99% of light vs 60-70% for standard mirrors, for a bright, sharp, distortion-free image with no secondary reflection.</t>
-        </is>
-      </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>ATRAUMATIC RETRACTION, MORE LIGHT: The broad 34mm head spreads pressure for comfortable cheek and tongue retraction in oral surgery, periodontics and orthodontic checks, and bounces more operatory light into dark posterior regions.</t>
@@ -1489,16 +1489,16 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The ILLUCO Grand Dental Mirror scales the standard mouth mirror up to a Size 10 (34mm) head, giving a 2.4x wider field of view than a standard Size 4 (22mm) mirror. View an entire quadrant, multi-unit restorations or full-arch alignment in a single glance and spend less time repositioning. The wide 34mm surface also distributes pressure evenly for comfortable cheek and tongue retraction, and works as a reflector that bounces more overhead light into deep posterior regions. ILLUCO's front surface dielectric coating on German optical glass reflects 99% of available light, compared with 60-70% for standard mirrors, and eliminates the ghost images that cause visual fatigue. The surface is large and distortion-free enough for clean quadrant photos. A water-repellent coating keeps the view clear mid-procedure, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each kit includes 2 Grand Size 10 mirror heads, 2 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in 1X and 2X magnification, Light Blue and Dark Blue.</t>
+          <t>The first thing dental professionals notice about an ILLUCO mirror is the view. Most dental mirrors reflect only 60-70% of available light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, so the image is over 40% brighter, sharp, true to color and free of the ghost images that cause visual fatigue. You see the difference the moment you look into it. The ILLUCO Grand Dental Mirror puts that clarity on a Size 10 (34mm) head, giving a 2.4x wider field of view than a standard Size 4 (22mm) mirror. View an entire quadrant, multi-unit restorations or full-arch alignment in a single glance and spend less time repositioning. The wide 34mm surface also distributes pressure evenly for comfortable cheek and tongue retraction, and works as a reflector that bounces more overhead light into deep posterior regions. The surface is large and distortion-free enough for clean quadrant photos. A water-repellent coating keeps the view clear mid-procedure, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each kit includes 2 Grand Size 10 mirror heads, 2 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in 1X and 2X magnification, Light Blue and Dark Blue.</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>large mouth mirror oversize jumbo wide view dentist orthodontist oral surgery retractor intraoral photography quadrant dental tools dentist instruments tooth teeth oral exam anti fog hygienist magnifying 2x</t>
+          <t>large mouth mirror oversize jumbo wide view dentist orthodontist oral surgery retractor intraoral photography quadrant dental tools dentist instruments tooth teeth oral exam anti fog hygienist magnifying 2x hd high definition</t>
         </is>
       </c>
       <c r="K6" s="3" t="n">
-        <v>206</v>
+        <v>225</v>
       </c>
     </row>
     <row r="7">
@@ -1509,20 +1509,20 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>ILLUCO Double-Sided Dental Mirror Size 4 (22mm) with Handles, 5 Pack, Front Surface Mouth Mirror, 99% Reflectance Both Sides, Fog-Resistant, Autoclavable 100X, No Ghost Image (1X, Light Blue)</t>
+          <t>ILLUCO Double-Sided UHD Dental Mirror Size 4 (22mm) with Handles, 5 Pack, Front Surface Mouth Mirror, 99% Reflectance Both Sides, Fog-Resistant, Autoclavable 100X, No Ghost Image (1X, Light Blue)</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>TWO MIRROR FACES, NO FLIPPING: Dielectric coating on both faces gives 99% reflectance on each side, so you can retract tissue with one face and view with the other without turning the mirror mid-procedure.</t>
+          <t>SEE THE DIFFERENCE AT FIRST LOOK: Most dental mirrors reflect only 60-70% of light, rhodium 80-85%. ILLUCO's UHD dielectric coating on German optical glass reflects 99% on BOTH faces, for an image over 40% brighter, crisp, true to color and free of ghosting. Look into it once and you will notice it.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>99% REFLECTANCE, ZERO GHOST IMAGES: Front surface dielectric coating on German optical glass reflects 99% of light vs 60-70% for standard mirrors and 80-85% for rhodium, for a brighter, sharper image with no secondary reflection.</t>
+          <t>TWO MIRROR FACES, NO FLIPPING: Retract tissue with one face and view with the other without turning the mirror mid-procedure. Both sides carry the same 99% UHD coating, so there is no weaker side.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1542,16 +1542,16 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The ILLUCO Double-Sided Dental Mirror brings ILLUCO's dielectric optical technology to a dual-sided format with 99% reflectance on both faces. Retract tissue with one side and view with the other, without flipping the mirror mid-procedure. Standard dental mirrors reflect 60-70% of available light and rhodium-coated mirrors reach 80-85%. ILLUCO's front surface dielectric coating on German optical glass reflects 99%, for a brighter, sharper image without the ghosting that causes visual fatigue during long procedures. At Size 4 (22mm) with a true 1X view, it suits routine exams, restorative checks, indirect vision and intraoral photography. A water-repellent coating keeps the view clear, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each pack includes 5 double-sided Size 4 mirror heads, 5 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in Light Blue and Dark Blue.</t>
+          <t>The first thing dental professionals notice about an ILLUCO mirror is the view. Most dental mirrors reflect only 60-70% of available light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, so the image is over 40% brighter, sharp, true to color and free of the ghost images that cause visual fatigue. You see the difference the moment you look into it. The ILLUCO Double-Sided Dental Mirror puts that clarity on both faces, so you can retract tissue with one side and view with the other without flipping the mirror mid-procedure. At Size 4 (22mm) with a true 1X view, it suits routine exams, restorative checks, indirect vision and intraoral photography. A water-repellent coating keeps the view clear, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each pack includes 5 double-sided Size 4 mirror heads, 5 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in Light Blue and Dark Blue.</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>two sided mouth mirror dual dentist tools dental instruments tooth teeth oral exam intraoral photography hygienist anti fog cone socket rhodium alternative number 4 professional dentist mirror for inside mouth</t>
+          <t>two sided mouth mirror dual dentist tools dental instruments tooth teeth oral exam intraoral photography hygienist anti fog cone socket rhodium alternative number 4 professional dentist mirror for inside mouth hd high definition</t>
         </is>
       </c>
       <c r="K7" s="3" t="n">
-        <v>209</v>
+        <v>228</v>
       </c>
     </row>
     <row r="8">
@@ -1562,20 +1562,20 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>ILLUCO Double-Sided Dental Mirror Size 4 (22mm) with Handles, 5 Pack, Front Surface Mouth Mirror, 99% Reflectance Both Sides, Fog-Resistant, Autoclavable 100X, No Ghost Image (1X, Dark Blue)</t>
+          <t>ILLUCO Double-Sided UHD Dental Mirror Size 4 (22mm) with Handles, 5 Pack, Front Surface Mouth Mirror, 99% Reflectance Both Sides, Fog-Resistant, Autoclavable 100X, No Ghost Image (1X, Dark Blue)</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>TWO MIRROR FACES, NO FLIPPING: Dielectric coating on both faces gives 99% reflectance on each side, so you can retract tissue with one face and view with the other without turning the mirror mid-procedure.</t>
+          <t>SEE THE DIFFERENCE AT FIRST LOOK: Most dental mirrors reflect only 60-70% of light, rhodium 80-85%. ILLUCO's UHD dielectric coating on German optical glass reflects 99% on BOTH faces, for an image over 40% brighter, crisp, true to color and free of ghosting. Look into it once and you will notice it.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>99% REFLECTANCE, ZERO GHOST IMAGES: Front surface dielectric coating on German optical glass reflects 99% of light vs 60-70% for standard mirrors and 80-85% for rhodium, for a brighter, sharper image with no secondary reflection.</t>
+          <t>TWO MIRROR FACES, NO FLIPPING: Retract tissue with one face and view with the other without turning the mirror mid-procedure. Both sides carry the same 99% UHD coating, so there is no weaker side.</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -1595,16 +1595,16 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The ILLUCO Double-Sided Dental Mirror brings ILLUCO's dielectric optical technology to a dual-sided format with 99% reflectance on both faces. Retract tissue with one side and view with the other, without flipping the mirror mid-procedure. Standard dental mirrors reflect 60-70% of available light and rhodium-coated mirrors reach 80-85%. ILLUCO's front surface dielectric coating on German optical glass reflects 99%, for a brighter, sharper image without the ghosting that causes visual fatigue during long procedures. At Size 4 (22mm) with a true 1X view, it suits routine exams, restorative checks, indirect vision and intraoral photography. A water-repellent coating keeps the view clear, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each pack includes 5 double-sided Size 4 mirror heads, 5 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in Light Blue and Dark Blue.</t>
+          <t>The first thing dental professionals notice about an ILLUCO mirror is the view. Most dental mirrors reflect only 60-70% of available light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, so the image is over 40% brighter, sharp, true to color and free of the ghost images that cause visual fatigue. You see the difference the moment you look into it. The ILLUCO Double-Sided Dental Mirror puts that clarity on both faces, so you can retract tissue with one side and view with the other without flipping the mirror mid-procedure. At Size 4 (22mm) with a true 1X view, it suits routine exams, restorative checks, indirect vision and intraoral photography. A water-repellent coating keeps the view clear, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each pack includes 5 double-sided Size 4 mirror heads, 5 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in Light Blue and Dark Blue.</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>two sided mouth mirror dual dentist tools dental instruments tooth teeth oral exam intraoral photography hygienist anti fog cone socket rhodium alternative number 4 professional dentist mirror for inside mouth</t>
+          <t>two sided mouth mirror dual dentist tools dental instruments tooth teeth oral exam intraoral photography hygienist anti fog cone socket rhodium alternative number 4 professional dentist mirror for inside mouth hd high definition</t>
         </is>
       </c>
       <c r="K8" s="3" t="n">
-        <v>209</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Apply master product sheet data to ILLUCO mirror upload file
- Prices: Retail Price from the master sheet as Your Price and List
  Price ($124 Grand 1X, $129 Grand 2X, $179 Double-Sided)
- Box: 8.27 x 3.94 x 1.38 in, 0.51 lb for all six SKUs
- Double-Sided Dark Blue uses the Light Blue main image for now
- Notes checklist updated: UPCs still open (empty in the master sheet),
  FDA fields pending, DS Light Blue shows no on-hand qty

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JtZ82rKJM1p58HzVJpKZqv
</commit_message>
<xml_diff>
--- a/CRL DOC/ILLUCO/ILLUCO_Upload_Notes.xlsx
+++ b/CRL DOC/ILLUCO/ILLUCO_Upload_Notes.xlsx
@@ -497,227 +497,227 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>No barcodes exist yet for these 6 SKUs (illuco.com has none). Existing ILLUCO kits use GS1 UPCs 81019486xxxx. Get 6 new UPCs, or set col J to 'GTIN Exempt' if ILLUCO has a GTIN exemption.</t>
+          <t>Still open: the Master Product Sheet's UPC column is empty for all 6 SKUs. Existing ILLUCO items use GS1 UPCs 81019486xxxx. Add 6 UPCs, or set col J to 'GTIN Exempt' if ILLUCO has a GTIN exemption.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>MUST</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
+          <t>FDA fields</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Template GU-GZ, rows 9-14</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Being confirmed by the team. Currently carried over from the ILLUCO profile: Class I, OTC, Consumer label, Professional instructions, 510(k) NULL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Double-Sided Light Blue stock</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Row 13 (IDM-2CD41LB)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Master sheet shows no on-hand qty for this SKU (Dark Blue has 250). Kept in the file; with FBA it just shows out of stock until a shipment arrives. Delete row 13 if it should not be listed yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
           <t>Main image for Double-Sided Dark Blue</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Template T14</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>illuco.com has no dark-blue Double-Sided photo. Add the URL, or upload it from S:\Ashley D\ILLUCO\Amazon\Double-Sided Dental Mirrors in Seller Central after the upload.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>MUST</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Measure box size and weight</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Uses the Light Blue photo for now, as agreed. Swap in a dark-blue photo when it exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Box size and weight</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Template EO-EV, rows 9-14</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Estimates: 9.5 x 4.5 x 1.5 in. Weight: Grand 1.0 lb (estimate), Double-Sided 2.0 lb (illuco.com shipping weight). FBA fees use these until Amazon re-measures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>CHECK</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>From the master sheet: 8.27 x 3.94 x 1.38 in (210 x 100 x 35 mm), 0.51 lb (sheet value 0.50485, read as pounds). Same box for all 6 SKUs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Country of origin</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Template EZ, all rows</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Set to 'Republic of Korea'. The template's saved Preference Profile had "Democratic People's Republic of Korea" (North Korea) - fix that profile in Seller Central too.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>CHECK</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Republic of Korea. Also fix the Seller Central Preference Profile, which had "Democratic People's Republic of Korea" (North Korea).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Prices</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Template DI</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Grand 1X $134, Grand 2X $139, Double-Sided $189 = illuco.com ($124 / $129 / $179) + $10, the same gap the live ILLUCO kits have on Amazon ($95/$125/$140 vs $85/$115/$130).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>CHECK</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Template DI (Your Price) and CF (List Price)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Master sheet Retail Price: Grand 1X $124, Grand 2X $129, Double-Sided $179. MAP is $99.20 / $103.20 / $143.20 - don't price or discount below it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Pack contents</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Titles, bullets, BM, AY</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Used the live illuco.com pages: Grand = 2 heads + 2 handles (2 Pack); Double-Sided = 5 heads + 5 handles (5 Pack). The launch-plan PDF said Grand 5 heads + 1 handle and DS 1 mirror + silicone sleeve; no sleeve is claimed in the listing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>CHECK</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Colors in stock</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Rows 9-14</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>illuco.com only sells Grand 1X Blue, Grand 2X Dark Blue and DS Blue today. You said both colors for all three sizes, so all 6 combinations are listed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>CHECK</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Matches the master sheet: Grand 2 units/box, Double-Sided 5 units/box, handles included.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>One variation family</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Rows 8-14</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>All 6 children sit under one parent (COLOR/SIZE) as '3 sizes x 2 colors', so reviews pool. If Amazon rejects mixing Grand and Double-Sided, give rows 13-14 their own parent row.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>CHECK</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>SKUs</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Template A, E, P, BC</t>
-        </is>
-      </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Follow the illuco.com SKU pattern (IDM-2C101LB = Grand, size 10, 1X, Light Blue; IDM-2CD41LB = Double-Sided, size 4, 1X). Confirm none already exist in Seller Central.</t>
+          <t>1 parent (IDM-GRAND-DS-PARENT) + 6 children, variation theme COLOR/SIZE.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Fulfillment</t>
+          <t>SKUs</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Template DD</t>
+          <t>Template A, E, P, BC</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Fulfillment by Amazon, like the existing ILLUCO 5-pack kits. Create the inbound shipment after the listings go live; quantity stays blank for FBA.</t>
+          <t>Match the master sheet exactly: IDM-2C101LB/DB, IDM-2C102LB/DB, IDM-2CD41LB/DB.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>FDA fields</t>
+          <t>Fulfillment</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Template GU-GZ</t>
+          <t>Template DD</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Carried over from your ILLUCO profile: Class I, OTC, Consumer label, Professional instructions, 510(k) NULL.</t>
+          <t>Fulfillment by Amazon (NA). Quantity stays blank; inventory arrives through an FBA shipment.</t>
         </is>
       </c>
     </row>
@@ -734,12 +734,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>CF, CG, DR, BL</t>
+          <t>CG, DR, BL, H</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>List price, tax code (account default applies), B2B price and launch date.</t>
+          <t>Tax code (account default applies), B2B price, launch date, item highlight.</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Catalog &gt; Add Products via Upload &gt; upload this .xlsm as is &gt; check the Processing Report.</t>
+          <t>1) Catalog &gt; Add Products via Upload &gt; 'Upload your spreadsheet'. 2) Choose this .xlsm as is (don't re-save it as .xlsx or .csv). 3) Wait for the Processing Report (often 15-60 min) and fix any errors it lists. 4) Inventory &gt; Manage All Inventory: confirm 1 parent + 6 children grouped. 5) Send to Amazon: create the FBA shipment and print FNSKU labels.</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -786,10 +786,12 @@
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="36" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="70" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="70" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -830,22 +832,32 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Amazon price $</t>
+          <t>Price = List $</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>illuco.com $</t>
+          <t>MAP $</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>On hand</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>UPC (fill in)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Main image URL</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Image note</t>
         </is>
       </c>
     </row>
@@ -869,6 +881,8 @@
       <c r="I2" s="3" t="inlineStr"/>
       <c r="J2" s="3" t="inlineStr"/>
       <c r="K2" s="3" t="inlineStr"/>
+      <c r="L2" s="3" t="inlineStr"/>
+      <c r="M2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -905,17 +919,21 @@
         <v>2</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>124</v>
-      </c>
-      <c r="J3" s="3" t="inlineStr"/>
-      <c r="K3" s="3" t="inlineStr">
+        <v>99.2</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="K3" s="3" t="inlineStr"/>
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0795/1348/5611/files/main_1b36fb35-6c34-4a82-81aa-68ef89447d58.jpg</t>
         </is>
       </c>
+      <c r="M3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -952,17 +970,21 @@
         <v>2</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>124</v>
-      </c>
-      <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr">
+        <v>99.2</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="K4" s="3" t="inlineStr"/>
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0795/1348/5611/files/main_db.jpg</t>
         </is>
       </c>
+      <c r="M4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -999,17 +1021,21 @@
         <v>2</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>129</v>
-      </c>
-      <c r="J5" s="3" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr">
+        <v>103.2</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="K5" s="3" t="inlineStr"/>
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0795/1348/5611/files/main_1b36fb35-6c34-4a82-81aa-68ef89447d58.jpg</t>
         </is>
       </c>
+      <c r="M5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1046,17 +1072,21 @@
         <v>2</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>129</v>
-      </c>
-      <c r="J6" s="3" t="inlineStr"/>
-      <c r="K6" s="3" t="inlineStr">
+        <v>103.2</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="K6" s="3" t="inlineStr"/>
+      <c r="L6" s="3" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0795/1348/5611/files/main_db.jpg</t>
         </is>
       </c>
+      <c r="M6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1093,17 +1123,23 @@
         <v>5</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>179</v>
-      </c>
-      <c r="J7" s="3" t="inlineStr"/>
-      <c r="K7" s="3" t="inlineStr">
+        <v>143.2</v>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>blank</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0795/1348/5611/files/main.jpg</t>
         </is>
       </c>
+      <c r="M7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1140,15 +1176,23 @@
         <v>5</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>179</v>
-      </c>
-      <c r="J8" s="3" t="inlineStr"/>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>MISSING - add dark blue DS photo</t>
+        <v>143.2</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="K8" s="3" t="inlineStr"/>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>https://cdn.shopify.com/s/files/1/0795/1348/5611/files/main.jpg</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>Light Blue photo used for now</t>
         </is>
       </c>
     </row>
@@ -3790,7 +3834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -3818,105 +3862,118 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>illuco.com - Grand Dental Mirror (Size 10) 2 Pack</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>https://illuco.com/products/grand-dental-mirror</t>
-        </is>
-      </c>
+          <t>Team 2026 ILLUCO Master Product Sheet (tier prices), 'Illuco' tab</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr"/>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Firecrawl + Shopify JSON: price $124 (1X) / $129 (2X), kit contents, SKUs, images</t>
+          <t>SKUs, Retail Price, MAP, on-hand qty, box size and weight, pack contents (UPC column empty)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>illuco.com - Double-Sided Dental Mirror (Size 4) 5 pack</t>
+          <t>illuco.com - Grand Dental Mirror (Size 10) 2 Pack</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>https://illuco.com/products/double-sided-dental-mirror</t>
+          <t>https://illuco.com/products/grand-dental-mirror</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Firecrawl + Shopify JSON: price $179, kit contents, SKU IDM-2CD41LB, 2.0 lb, images</t>
+          <t>Firecrawl + Shopify JSON: price $124 (1X) / $129 (2X), kit contents, SKUs, images</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>illuco.com - Dental Mirror Kit (Size 4)</t>
+          <t>illuco.com - Double-Sided Dental Mirror (Size 4) 5 pack</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>https://illuco.com/products/dental-mirror</t>
+          <t>https://illuco.com/products/double-sided-dental-mirror</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Shopify JSON: SKU pattern IDM-2C41DB and existing UPCs 81019486xxxx</t>
+          <t>Firecrawl + Shopify JSON: price $179, kit contents, SKU IDM-2CD41LB, 2.0 lb, images</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Amazon search via Apify (automly/amazon-products-scraper)</t>
+          <t>illuco.com - Dental Mirror Kit (Size 4)</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/s?k=ILLUCO+dental+mirror</t>
+          <t>https://illuco.com/products/dental-mirror</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Existing ILLUCO USA listings, prices, reviews, BSR; competitor sets for 'double sided dental mirror' and 'large dental mirror' (scraped 2026-10-28)</t>
+          <t>Shopify JSON: SKU pattern IDM-2C41DB and existing UPCs 81019486xxxx</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>ILLUCO Sales &amp; Marketing Launch Plan (PDF)</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr"/>
+          <t>Amazon search via Apify (automly/amazon-products-scraper)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/s?k=ILLUCO+dental+mirror</t>
+        </is>
+      </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Positioning, claims, keyword table</t>
+          <t>Existing ILLUCO USA listings, prices, reviews, BSR; competitor sets for 'double sided dental mirror' and 'large dental mirror' (scraped 2026-10-28)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>ILLUCO Dental Mirror Market Intelligence Report (PDF)</t>
+          <t>ILLUCO Sales &amp; Marketing Launch Plan (PDF)</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr"/>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Pricing principles, competitor gaps</t>
+          <t>Positioning, claims, keyword table</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Vic - Dental Mirror Keyword sheet</t>
+          <t>ILLUCO Dental Mirror Market Intelligence Report (PDF)</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr"/>
       <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Pricing principles, competitor gaps</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Vic - Dental Mirror Keyword sheet</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Search volumes used for backend keywords</t>
         </is>

</xml_diff>

<commit_message>
Use Amazon item name + item highlight format for ILLUCO mirrors
- Item names cut to 62-72 characters so Amazon shows the Item
  Highlight (it only displays when the name is under 75 characters)
- Item Highlight (col H) carries the benefit phrases
- Package Level (col M) = Unit on all six children
- Double-Sided Light Blue marked in stock in the notes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JtZ82rKJM1p58HzVJpKZqv
</commit_message>
<xml_diff>
--- a/CRL DOC/ILLUCO/ILLUCO_Upload_Notes.xlsx
+++ b/CRL DOC/ILLUCO/ILLUCO_Upload_Notes.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -524,9 +524,9 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>CHECK</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -541,7 +541,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Master sheet shows no on-hand qty for this SKU (Dark Blue has 250). Kept in the file; with FBA it just shows out of stock until a shipment arrives. Delete row 13 if it should not be listed yet.</t>
+          <t>In stock (confirmed by the team; the master sheet's on-hand cell is blank).</t>
         </is>
       </c>
     </row>
@@ -553,17 +553,17 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Main image for Double-Sided Dark Blue</t>
+          <t>Item name + item highlight</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Template T14</t>
+          <t>Template G and H, all rows</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Uses the Light Blue photo for now, as agreed. Swap in a dark-blue photo when it exists.</t>
+          <t>Short item names (62-72 characters) so the Item Highlight shows; Amazon only displays the highlight when the name is under 75 characters. Highlights carry the benefit phrases, not repeated in the name.</t>
         </is>
       </c>
     </row>
@@ -575,17 +575,17 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Box size and weight</t>
+          <t>Package level</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Template EO-EV, rows 9-14</t>
+          <t>Template M, rows 9-14</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>From the master sheet: 8.27 x 3.94 x 1.38 in (210 x 100 x 35 mm), 0.51 lb (sheet value 0.50485, read as pounds). Same box for all 6 SKUs.</t>
+          <t>'Unit': each SKU is one retail box sold on its own. 'Case'/'Pallet' are only for a separate case-pack SKU (e.g. 10 boxes), which then needs Package Contains SKU Quantity/Identifier (N, O).</t>
         </is>
       </c>
     </row>
@@ -597,17 +597,17 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Country of origin</t>
+          <t>Main image for Double-Sided Dark Blue</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Template EZ, all rows</t>
+          <t>Template T14</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Republic of Korea. Also fix the Seller Central Preference Profile, which had "Democratic People's Republic of Korea" (North Korea).</t>
+          <t>Uses the Light Blue photo for now, as agreed. Swap in a dark-blue photo when it exists.</t>
         </is>
       </c>
     </row>
@@ -619,17 +619,17 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Prices</t>
+          <t>Box size and weight</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Template DI (Your Price) and CF (List Price)</t>
+          <t>Template EO-EV, rows 9-14</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Master sheet Retail Price: Grand 1X $124, Grand 2X $129, Double-Sided $179. MAP is $99.20 / $103.20 / $143.20 - don't price or discount below it.</t>
+          <t>From the master sheet: 8.27 x 3.94 x 1.38 in (210 x 100 x 35 mm), 0.51 lb (sheet value 0.50485, read as pounds). Same box for all 6 SKUs.</t>
         </is>
       </c>
     </row>
@@ -641,17 +641,17 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Pack contents</t>
+          <t>Country of origin</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Titles, bullets, BM, AY</t>
+          <t>Template EZ, all rows</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Matches the master sheet: Grand 2 units/box, Double-Sided 5 units/box, handles included.</t>
+          <t>Republic of Korea. Also fix the Seller Central Preference Profile, which had "Democratic People's Republic of Korea" (North Korea).</t>
         </is>
       </c>
     </row>
@@ -663,17 +663,17 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>One variation family</t>
+          <t>Prices</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Rows 8-14</t>
+          <t>Template DI (Your Price) and CF (List Price)</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>1 parent (IDM-GRAND-DS-PARENT) + 6 children, variation theme COLOR/SIZE.</t>
+          <t>Master sheet Retail Price: Grand 1X $124, Grand 2X $129, Double-Sided $179. MAP is $99.20 / $103.20 / $143.20 - don't price or discount below it.</t>
         </is>
       </c>
     </row>
@@ -685,17 +685,17 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SKUs</t>
+          <t>Pack contents</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Template A, E, P, BC</t>
+          <t>Titles, bullets, BM, AY</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Match the master sheet exactly: IDM-2C101LB/DB, IDM-2C102LB/DB, IDM-2CD41LB/DB.</t>
+          <t>Matches the master sheet: Grand 2 units/box, Double-Sided 5 units/box, handles included.</t>
         </is>
       </c>
     </row>
@@ -707,59 +707,103 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Fulfillment</t>
+          <t>One variation family</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Template DD</t>
+          <t>Rows 8-14</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Fulfillment by Amazon (NA). Quantity stays blank; inventory arrives through an FBA shipment.</t>
+          <t>1 parent (IDM-GRAND-DS-PARENT) + 6 children, variation theme COLOR/SIZE.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Left blank on purpose</t>
+          <t>SKUs</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>CG, DR, BL, H</t>
+          <t>Template A, E, P, BC</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Tax code (account default applies), B2B price, launch date, item highlight.</t>
+          <t>Match the master sheet exactly: IDM-2C101LB/DB, IDM-2C102LB/DB, IDM-2CD41LB/DB.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Fulfillment</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Template DD</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Fulfillment by Amazon (NA). Quantity stays blank; inventory arrives through an FBA shipment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Left blank on purpose</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>CG, DR, BL, H</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Tax code (account default applies), B2B price, launch date, item highlight.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>How to upload</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Seller Central</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>1) Catalog &gt; Add Products via Upload &gt; 'Upload your spreadsheet'. 2) Choose this .xlsm as is (don't re-save it as .xlsx or .csv). 3) Wait for the Processing Report (often 15-60 min) and fix any errors it lists. 4) Inventory &gt; Manage All Inventory: confirm 1 parent + 6 children grouped. 5) Send to Amazon: create the FBA shipment and print FNSKU labels.</t>
         </is>
@@ -1130,7 +1174,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>blank</t>
+          <t>in stock (team confirmed)</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr"/>
@@ -1207,20 +1251,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
-    <col width="80" customWidth="1" min="9" max="9"/>
-    <col width="50" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="80" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1231,50 +1276,55 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Item name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Title chars (max 200)</t>
+          <t>Name chars (under 75)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Item highlight</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Bullet 1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Bullet 2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Bullet 3</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Bullet 4</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Bullet 5</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Backend keywords</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Keyword bytes (max 249)</t>
         </is>
@@ -1288,48 +1338,53 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>ILLUCO UHD Dental Mirrors with Handles, Grand Size 10 (34mm) and Double-Sided Size 4 (22mm), Front Surface Dielectric Mouth Mirror, 99% Reflectance, Fog-Resistant, Autoclavable 100X</t>
+          <t>ILLUCO UHD Dental Mirrors with Handles, Grand and Double-Sided</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>181</v>
+        <v>62</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
+          <t>99% Reflectance, Fog-Resistant, Autoclavable 100X, No Ghost Image</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
           <t>SEE THE DIFFERENCE AT FIRST LOOK: Most dental mirrors reflect only 60-70% of light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, for an image over 40% brighter, crisp, true to color and free of ghosting. Look into it once and you will notice it.</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>TWO NEW ILLUCO MIRRORS: Grand Size 10 (34mm) in 1X or 2X for a 2.4x wider field of view, and Double-Sided Size 4 (22mm) with 99% reflectance on both faces.</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>FOG-RESISTANT: Water-repellent coating sheds saliva and spray mid-procedure.</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>AUTOCLAVABLE 100X: Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C).</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>ERGONOMIC HANDLES INCLUDED: Anti-rotation handles in Light Blue or Dark Blue.</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>The first thing dental professionals notice about an ILLUCO mirror is the view. Most dental mirrors reflect only 60-70% of available light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, so the image is over 40% brighter, sharp, true to color and free of the ghost images that cause visual fatigue. You see the difference the moment you look into it. The fog-resistant, water-repellent surface withstands 100 autoclave cycles. Choose the Grand Size 10 (34mm) mirror in 1X or 2X for a 2.4x wider field of view, or the Double-Sided Size 4 (22mm) mirror with 99% reflectance on both faces. Each kit includes ergonomic anti-rotation handles in Light Blue or Dark Blue. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C).</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>mouth mirror dentist tools dental instruments tooth teeth oral exam intraoral photography hygienist orthodontist anti fog large double sided</t>
         </is>
       </c>
-      <c r="K2" s="3" t="n">
+      <c r="L2" s="3" t="n">
         <v>140</v>
       </c>
     </row>
@@ -1341,48 +1396,53 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>ILLUCO Grand UHD Dental Mirror Size 10 (34mm) with Handles, 2 Pack, Large Front Surface Mouth Mirror, 99% Reflectance, Fog-Resistant, Autoclavable 100X, No Ghost Image (1X, Light Blue)</t>
+          <t>ILLUCO Grand UHD Dental Mirror, Size 10 (34mm), 1X, 2 Pack, Light Blue</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>184</v>
+        <v>70</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
+          <t>With Handles, 99% Reflectance, 2.4X Wider View, Fog-Resistant, Autoclavable 100X, No Ghost Image</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
           <t>SEE THE DIFFERENCE AT FIRST LOOK: Most dental mirrors reflect only 60-70% of light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, for an image over 40% brighter, crisp, true to color and free of ghosting. Look into it once and you will notice it.</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>2.4X WIDER FIELD OF VIEW: The Size 10 (34mm) head covers 2.4 times the viewing area of a standard Size 4 (22mm) mirror. See a full quadrant, multi-unit restorations or the whole arch in one view, with far less mirror repositioning.</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>ATRAUMATIC RETRACTION, MORE LIGHT: The broad 34mm head spreads pressure for comfortable cheek and tongue retraction in oral surgery, periodontics and orthodontic checks, and bounces more operatory light into dark posterior regions.</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>FOG-RESISTANT AND AUTOCLAVABLE 100X: Water-repellent coating sheds saliva and spray mid-procedure. Glass and coating withstand 100 autoclave cycles without staining or losing reflectivity. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C).</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>KIT INCLUDES 2 MIRRORS WITH HANDLES: 2 Grand Size 10 mirror heads, 2 ergonomic anti-rotation handles (Light Blue) and an autoclave sterilization and care guide. 1X gives a true life-size, distortion-free view for exams and quadrant photography. Also available in 2X magnification and with Dark Blue handles.</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>The first thing dental professionals notice about an ILLUCO mirror is the view. Most dental mirrors reflect only 60-70% of available light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, so the image is over 40% brighter, sharp, true to color and free of the ghost images that cause visual fatigue. You see the difference the moment you look into it. The ILLUCO Grand Dental Mirror puts that clarity on a Size 10 (34mm) head, giving a 2.4x wider field of view than a standard Size 4 (22mm) mirror. View an entire quadrant, multi-unit restorations or full-arch alignment in a single glance and spend less time repositioning. The wide 34mm surface also distributes pressure evenly for comfortable cheek and tongue retraction, and works as a reflector that bounces more overhead light into deep posterior regions. The surface is large and distortion-free enough for clean quadrant photos. A water-repellent coating keeps the view clear mid-procedure, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each kit includes 2 Grand Size 10 mirror heads, 2 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in 1X and 2X magnification, Light Blue and Dark Blue.</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>large mouth mirror oversize jumbo wide view dentist orthodontist oral surgery retractor intraoral photography quadrant dental tools dentist instruments tooth teeth oral exam anti fog hygienist magnifying 2x hd high definition</t>
         </is>
       </c>
-      <c r="K3" s="3" t="n">
+      <c r="L3" s="3" t="n">
         <v>225</v>
       </c>
     </row>
@@ -1394,48 +1454,53 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>ILLUCO Grand UHD Dental Mirror Size 10 (34mm) with Handles, 2 Pack, Large Front Surface Mouth Mirror, 99% Reflectance, Fog-Resistant, Autoclavable 100X, No Ghost Image (1X, Dark Blue)</t>
+          <t>ILLUCO Grand UHD Dental Mirror, Size 10 (34mm), 1X, 2 Pack, Dark Blue</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>183</v>
+        <v>69</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
+          <t>With Handles, 99% Reflectance, 2.4X Wider View, Fog-Resistant, Autoclavable 100X, No Ghost Image</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
           <t>SEE THE DIFFERENCE AT FIRST LOOK: Most dental mirrors reflect only 60-70% of light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, for an image over 40% brighter, crisp, true to color and free of ghosting. Look into it once and you will notice it.</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>2.4X WIDER FIELD OF VIEW: The Size 10 (34mm) head covers 2.4 times the viewing area of a standard Size 4 (22mm) mirror. See a full quadrant, multi-unit restorations or the whole arch in one view, with far less mirror repositioning.</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>ATRAUMATIC RETRACTION, MORE LIGHT: The broad 34mm head spreads pressure for comfortable cheek and tongue retraction in oral surgery, periodontics and orthodontic checks, and bounces more operatory light into dark posterior regions.</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>FOG-RESISTANT AND AUTOCLAVABLE 100X: Water-repellent coating sheds saliva and spray mid-procedure. Glass and coating withstand 100 autoclave cycles without staining or losing reflectivity. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C).</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>KIT INCLUDES 2 MIRRORS WITH HANDLES: 2 Grand Size 10 mirror heads, 2 ergonomic anti-rotation handles (Dark Blue) and an autoclave sterilization and care guide. 1X gives a true life-size, distortion-free view for exams and quadrant photography. Also available in 2X magnification and with Light Blue handles.</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>The first thing dental professionals notice about an ILLUCO mirror is the view. Most dental mirrors reflect only 60-70% of available light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, so the image is over 40% brighter, sharp, true to color and free of the ghost images that cause visual fatigue. You see the difference the moment you look into it. The ILLUCO Grand Dental Mirror puts that clarity on a Size 10 (34mm) head, giving a 2.4x wider field of view than a standard Size 4 (22mm) mirror. View an entire quadrant, multi-unit restorations or full-arch alignment in a single glance and spend less time repositioning. The wide 34mm surface also distributes pressure evenly for comfortable cheek and tongue retraction, and works as a reflector that bounces more overhead light into deep posterior regions. The surface is large and distortion-free enough for clean quadrant photos. A water-repellent coating keeps the view clear mid-procedure, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each kit includes 2 Grand Size 10 mirror heads, 2 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in 1X and 2X magnification, Light Blue and Dark Blue.</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>large mouth mirror oversize jumbo wide view dentist orthodontist oral surgery retractor intraoral photography quadrant dental tools dentist instruments tooth teeth oral exam anti fog hygienist magnifying 2x hd high definition</t>
         </is>
       </c>
-      <c r="K4" s="3" t="n">
+      <c r="L4" s="3" t="n">
         <v>225</v>
       </c>
     </row>
@@ -1447,48 +1512,53 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>ILLUCO Grand UHD Dental Mirror Size 10 (34mm) with Handles, 2 Pack, Large Front Surface Mouth Mirror, 99% Reflectance, Fog-Resistant, Autoclavable 100X, No Ghost Image (2X, Light Blue)</t>
+          <t>ILLUCO Grand UHD Dental Mirror, Size 10 (34mm), 2X, 2 Pack, Light Blue</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>184</v>
+        <v>70</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
+          <t>With Handles, 99% Reflectance, 2.4X Wider View, Fog-Resistant, Autoclavable 100X, No Ghost Image</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
           <t>SEE THE DIFFERENCE AT FIRST LOOK: Most dental mirrors reflect only 60-70% of light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, for an image over 40% brighter, crisp, true to color and free of ghosting. Look into it once and you will notice it.</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>2.4X WIDER FIELD OF VIEW: The Size 10 (34mm) head covers 2.4 times the viewing area of a standard Size 4 (22mm) mirror. See a full quadrant, multi-unit restorations or the whole arch in one view, with far less mirror repositioning.</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>ATRAUMATIC RETRACTION, MORE LIGHT: The broad 34mm head spreads pressure for comfortable cheek and tongue retraction in oral surgery, periodontics and orthodontic checks, and bounces more operatory light into dark posterior regions.</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>FOG-RESISTANT AND AUTOCLAVABLE 100X: Water-repellent coating sheds saliva and spray mid-procedure. Glass and coating withstand 100 autoclave cycles without staining or losing reflectivity. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C).</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>KIT INCLUDES 2 MIRRORS WITH HANDLES: 2 Grand Size 10 mirror heads, 2 ergonomic anti-rotation handles (Light Blue) and an autoclave sterilization and care guide. 2X magnification enlarges margins and fine detail across the wide 34mm field. Also available in 1X magnification and with Dark Blue handles.</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>The first thing dental professionals notice about an ILLUCO mirror is the view. Most dental mirrors reflect only 60-70% of available light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, so the image is over 40% brighter, sharp, true to color and free of the ghost images that cause visual fatigue. You see the difference the moment you look into it. The ILLUCO Grand Dental Mirror puts that clarity on a Size 10 (34mm) head, giving a 2.4x wider field of view than a standard Size 4 (22mm) mirror. View an entire quadrant, multi-unit restorations or full-arch alignment in a single glance and spend less time repositioning. The wide 34mm surface also distributes pressure evenly for comfortable cheek and tongue retraction, and works as a reflector that bounces more overhead light into deep posterior regions. The surface is large and distortion-free enough for clean quadrant photos. A water-repellent coating keeps the view clear mid-procedure, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each kit includes 2 Grand Size 10 mirror heads, 2 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in 1X and 2X magnification, Light Blue and Dark Blue.</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>large mouth mirror oversize jumbo wide view dentist orthodontist oral surgery retractor intraoral photography quadrant dental tools dentist instruments tooth teeth oral exam anti fog hygienist magnifying 2x hd high definition</t>
         </is>
       </c>
-      <c r="K5" s="3" t="n">
+      <c r="L5" s="3" t="n">
         <v>225</v>
       </c>
     </row>
@@ -1500,48 +1570,53 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>ILLUCO Grand UHD Dental Mirror Size 10 (34mm) with Handles, 2 Pack, Large Front Surface Mouth Mirror, 99% Reflectance, Fog-Resistant, Autoclavable 100X, No Ghost Image (2X, Dark Blue)</t>
+          <t>ILLUCO Grand UHD Dental Mirror, Size 10 (34mm), 2X, 2 Pack, Dark Blue</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>183</v>
+        <v>69</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
+          <t>With Handles, 99% Reflectance, 2.4X Wider View, Fog-Resistant, Autoclavable 100X, No Ghost Image</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
           <t>SEE THE DIFFERENCE AT FIRST LOOK: Most dental mirrors reflect only 60-70% of light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, for an image over 40% brighter, crisp, true to color and free of ghosting. Look into it once and you will notice it.</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>2.4X WIDER FIELD OF VIEW: The Size 10 (34mm) head covers 2.4 times the viewing area of a standard Size 4 (22mm) mirror. See a full quadrant, multi-unit restorations or the whole arch in one view, with far less mirror repositioning.</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>ATRAUMATIC RETRACTION, MORE LIGHT: The broad 34mm head spreads pressure for comfortable cheek and tongue retraction in oral surgery, periodontics and orthodontic checks, and bounces more operatory light into dark posterior regions.</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>FOG-RESISTANT AND AUTOCLAVABLE 100X: Water-repellent coating sheds saliva and spray mid-procedure. Glass and coating withstand 100 autoclave cycles without staining or losing reflectivity. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C).</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>KIT INCLUDES 2 MIRRORS WITH HANDLES: 2 Grand Size 10 mirror heads, 2 ergonomic anti-rotation handles (Dark Blue) and an autoclave sterilization and care guide. 2X magnification enlarges margins and fine detail across the wide 34mm field. Also available in 1X magnification and with Light Blue handles.</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>The first thing dental professionals notice about an ILLUCO mirror is the view. Most dental mirrors reflect only 60-70% of available light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, so the image is over 40% brighter, sharp, true to color and free of the ghost images that cause visual fatigue. You see the difference the moment you look into it. The ILLUCO Grand Dental Mirror puts that clarity on a Size 10 (34mm) head, giving a 2.4x wider field of view than a standard Size 4 (22mm) mirror. View an entire quadrant, multi-unit restorations or full-arch alignment in a single glance and spend less time repositioning. The wide 34mm surface also distributes pressure evenly for comfortable cheek and tongue retraction, and works as a reflector that bounces more overhead light into deep posterior regions. The surface is large and distortion-free enough for clean quadrant photos. A water-repellent coating keeps the view clear mid-procedure, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each kit includes 2 Grand Size 10 mirror heads, 2 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in 1X and 2X magnification, Light Blue and Dark Blue.</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>large mouth mirror oversize jumbo wide view dentist orthodontist oral surgery retractor intraoral photography quadrant dental tools dentist instruments tooth teeth oral exam anti fog hygienist magnifying 2x hd high definition</t>
         </is>
       </c>
-      <c r="K6" s="3" t="n">
+      <c r="L6" s="3" t="n">
         <v>225</v>
       </c>
     </row>
@@ -1553,48 +1628,53 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>ILLUCO Double-Sided UHD Dental Mirror Size 4 (22mm) with Handles, 5 Pack, Front Surface Mouth Mirror, 99% Reflectance Both Sides, Fog-Resistant, Autoclavable 100X, No Ghost Image (1X, Light Blue)</t>
+          <t>ILLUCO Double-Sided UHD Dental Mirror, Size 4 (22mm), 5 Pack, Light Blue</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>195</v>
+        <v>72</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
+          <t>With Handles, 1X, 99% Reflectance Both Sides, Fog-Resistant, Autoclavable 100X, No Ghost Image</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
           <t>SEE THE DIFFERENCE AT FIRST LOOK: Most dental mirrors reflect only 60-70% of light, rhodium 80-85%. ILLUCO's UHD dielectric coating on German optical glass reflects 99% on BOTH faces, for an image over 40% brighter, crisp, true to color and free of ghosting. Look into it once and you will notice it.</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>TWO MIRROR FACES, NO FLIPPING: Retract tissue with one face and view with the other without turning the mirror mid-procedure. Both sides carry the same 99% UHD coating, so there is no weaker side.</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>STANDARD SIZE 4 (22MM), TRUE 1X VIEW: Life-size, distortion-free reflection for routine exams, restorative checks, indirect vision and intraoral photography. The ergonomic anti-rotation handle keeps the head steady in your grip.</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>FOG-RESISTANT AND AUTOCLAVABLE 100X: Water-repellent coating sheds saliva and spray mid-procedure. Glass and coating withstand 100 autoclave cycles without staining or losing reflectivity. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C).</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>5 PACK WITH HANDLES: 5 double-sided Size 4 mirror heads, 5 ergonomic anti-rotation handles (Light Blue) and an autoclave sterilization and care guide. Built for general dentists, hygienists, orthodontists and dental photographers.</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>The first thing dental professionals notice about an ILLUCO mirror is the view. Most dental mirrors reflect only 60-70% of available light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, so the image is over 40% brighter, sharp, true to color and free of the ghost images that cause visual fatigue. You see the difference the moment you look into it. The ILLUCO Double-Sided Dental Mirror puts that clarity on both faces, so you can retract tissue with one side and view with the other without flipping the mirror mid-procedure. At Size 4 (22mm) with a true 1X view, it suits routine exams, restorative checks, indirect vision and intraoral photography. A water-repellent coating keeps the view clear, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each pack includes 5 double-sided Size 4 mirror heads, 5 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in Light Blue and Dark Blue.</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>two sided mouth mirror dual dentist tools dental instruments tooth teeth oral exam intraoral photography hygienist anti fog cone socket rhodium alternative number 4 professional dentist mirror for inside mouth hd high definition</t>
         </is>
       </c>
-      <c r="K7" s="3" t="n">
+      <c r="L7" s="3" t="n">
         <v>228</v>
       </c>
     </row>
@@ -1606,48 +1686,53 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>ILLUCO Double-Sided UHD Dental Mirror Size 4 (22mm) with Handles, 5 Pack, Front Surface Mouth Mirror, 99% Reflectance Both Sides, Fog-Resistant, Autoclavable 100X, No Ghost Image (1X, Dark Blue)</t>
+          <t>ILLUCO Double-Sided UHD Dental Mirror, Size 4 (22mm), 5 Pack, Dark Blue</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>194</v>
+        <v>71</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
+          <t>With Handles, 1X, 99% Reflectance Both Sides, Fog-Resistant, Autoclavable 100X, No Ghost Image</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
           <t>SEE THE DIFFERENCE AT FIRST LOOK: Most dental mirrors reflect only 60-70% of light, rhodium 80-85%. ILLUCO's UHD dielectric coating on German optical glass reflects 99% on BOTH faces, for an image over 40% brighter, crisp, true to color and free of ghosting. Look into it once and you will notice it.</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>TWO MIRROR FACES, NO FLIPPING: Retract tissue with one face and view with the other without turning the mirror mid-procedure. Both sides carry the same 99% UHD coating, so there is no weaker side.</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>STANDARD SIZE 4 (22MM), TRUE 1X VIEW: Life-size, distortion-free reflection for routine exams, restorative checks, indirect vision and intraoral photography. The ergonomic anti-rotation handle keeps the head steady in your grip.</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>FOG-RESISTANT AND AUTOCLAVABLE 100X: Water-repellent coating sheds saliva and spray mid-procedure. Glass and coating withstand 100 autoclave cycles without staining or losing reflectivity. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C).</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>5 PACK WITH HANDLES: 5 double-sided Size 4 mirror heads, 5 ergonomic anti-rotation handles (Dark Blue) and an autoclave sterilization and care guide. Built for general dentists, hygienists, orthodontists and dental photographers.</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>The first thing dental professionals notice about an ILLUCO mirror is the view. Most dental mirrors reflect only 60-70% of available light. ILLUCO's UHD front surface dielectric coating on German optical glass reflects 99%, so the image is over 40% brighter, sharp, true to color and free of the ghost images that cause visual fatigue. You see the difference the moment you look into it. The ILLUCO Double-Sided Dental Mirror puts that clarity on both faces, so you can retract tissue with one side and view with the other without flipping the mirror mid-procedure. At Size 4 (22mm) with a true 1X view, it suits routine exams, restorative checks, indirect vision and intraoral photography. A water-repellent coating keeps the view clear, and the mirror withstands 100 autoclave cycles. Sterilize at 273°F (134°C) for 5 minutes or 250°F (121°C) for 20 minutes; do not exceed 277°F (136°C). Each pack includes 5 double-sided Size 4 mirror heads, 5 ergonomic anti-rotation handles and an autoclave sterilization and care guide. Available in Light Blue and Dark Blue.</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>two sided mouth mirror dual dentist tools dental instruments tooth teeth oral exam intraoral photography hygienist anti fog cone socket rhodium alternative number 4 professional dentist mirror for inside mouth hd high definition</t>
         </is>
       </c>
-      <c r="K8" s="3" t="n">
+      <c r="L8" s="3" t="n">
         <v>228</v>
       </c>
     </row>

</xml_diff>